<commit_message>
Report Generation - Test Cases + Screenshots + AI Vision
</commit_message>
<xml_diff>
--- a/test_cases/sample_test_cases.xlsx
+++ b/test_cases/sample_test_cases.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="540" windowWidth="23655" windowHeight="9915" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Test Cases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -522,7 +522,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) The booking reference element visibly contains the text 'BK-387717', which includes the required 'BK-' prefix.</t>
+          <t>[PASS] (PASS:1 FAIL:0 UNCERTAIN:0) The booking confirmation is clearly displayed with a booking reference (BK-420405) and summary details.</t>
         </is>
       </c>
     </row>
@@ -567,7 +567,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) The first room card for 'Grand Hotel' is clearly visible in the search results.</t>
+          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) The room price of $150 per night is clearly visible in a blue container on the right side of the page.</t>
+          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
         </is>
       </c>
     </row>
@@ -679,7 +679,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) The 'My Bookings' page is clearly visible, displaying a confirmed booking for Grand Hotel.</t>
+          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
         </is>
       </c>
     </row>
@@ -740,7 +740,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) The validation error message 'First name is required.' is clearly visible below the First Name input field.</t>
+          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) The validation error message 'Last name is required.' is clearly visible below the Last Name input field.</t>
+          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>[PASS] (PASS:2 FAIL:0 UNCERTAIN:0) The validation error message 'Please enter a valid email address.' is clearly visible below the email field.</t>
+          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>[UNCERTAIN] (PASS:1 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
+          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
         </is>
       </c>
     </row>
@@ -984,7 +984,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:2) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
+          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
         </is>
       </c>
     </row>
@@ -1045,7 +1045,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:2) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
+          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:2) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
+          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:2) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
+          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:2) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
+          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
         </is>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:2) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
+          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
         </is>
       </c>
     </row>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:2) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
+          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rate limit issue solved
</commit_message>
<xml_diff>
--- a/test_cases/sample_test_cases.xlsx
+++ b/test_cases/sample_test_cases.xlsx
@@ -522,7 +522,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>[PASS] (PASS:1 FAIL:0 UNCERTAIN:0) The booking confirmation is clearly displayed with a booking reference (BK-420405) and summary details.</t>
+          <t>[PASS] (PASS:1 FAIL:0 UNCERTAIN:0) Booking confirmation details and booking reference (BK-923198) are clearly displayed.</t>
         </is>
       </c>
     </row>
@@ -567,7 +567,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
+          <t>[PASS] (PASS:1 FAIL:0 UNCERTAIN:0) Available room cards featuring hotel titles, pricing, room types, amenities, and images are displayed.</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
+          <t>[PASS] (PASS:1 FAIL:0 UNCERTAIN:0) Room details including title, room type, image, price, description, and amenities are clearly displayed.</t>
         </is>
       </c>
     </row>
@@ -679,7 +679,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
+          <t>[PASS] (PASS:1 FAIL:0 UNCERTAIN:0) The 'My Bookings' page is displayed showing a confirmed booking for Grand Hotel.</t>
         </is>
       </c>
     </row>
@@ -740,7 +740,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
+          <t>[PASS] (PASS:1 FAIL:0 UNCERTAIN:0) A validation error message 'First name is required.' is clearly visible below the First Name field.</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
+          <t>[PASS] (PASS:1 FAIL:0 UNCERTAIN:0) A validation error message "Last name is required." is clearly visible below the Last Name field.</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
+          <t>[PASS] (PASS:1 FAIL:0 UNCERTAIN:0) A validation error message 'Please enter a valid email address.' is clearly visible below the email field.</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
+          <t>[PASS] (PASS:1 FAIL:0 UNCERTAIN:0) A validation error message 'Phone number must contain only digits.' is clearly visible below the Phone input field.</t>
         </is>
       </c>
     </row>
@@ -984,7 +984,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
+          <t>[PASS] (PASS:1 FAIL:0 UNCERTAIN:0) A validation error message 'Phone number must contain exactly 10 digits.' is clearly visible under the phone input field.</t>
         </is>
       </c>
     </row>
@@ -1045,7 +1045,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
+          <t>[PASS] (PASS:1 FAIL:0 UNCERTAIN:0) The validation error 'Check-out date must be after check-in date.' is clearly visible in red text below the check-out field.</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
+          <t>[PASS] (PASS:1 FAIL:0 UNCERTAIN:0) A validation error stating 'Number of guests must be between 1 and 10.' is clearly visible below the Number of Guests field.</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
+          <t>[PASS] (PASS:1 FAIL:0 UNCERTAIN:0) A validation error message stating 'Number of guests must be between 1 and 10' is clearly visible below the guests field.</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
+          <t>[PASS] (PASS:1 FAIL:0 UNCERTAIN:0) A validation error message stating 'Card number must contain exactly 16 digits.' is clearly visible below the card number field.</t>
         </is>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
+          <t>[PASS] (PASS:1 FAIL:0 UNCERTAIN:0) A validation error message reading 'Card has expired.' is clearly visible under the Expiry Date field.</t>
         </is>
       </c>
     </row>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>[UNCERTAIN] (PASS:0 FAIL:0 UNCERTAIN:1) AI quota exhausted (429). Reduce AI_VERIFY_EVERY_SCREENSHOT or wait for quota reset. model gemini-3-flash-preview: ClientError: 429 RESOURCE_EXHAUSTED. {'error': {'code': 429, 'message': 'You exceeded your current quota, please check your plan and billing details. For more information on this error, head to: https://ai.google.dev/gemini-api/docs/rate-limits. To m...</t>
+          <t>[PASS] (PASS:1 FAIL:0 UNCERTAIN:0) A validation error message 'CVV must contain exactly 3 digits.' is clearly visible below the CVV field.</t>
         </is>
       </c>
     </row>

</xml_diff>